<commit_message>
feature(hyperp_exploration): Re-do one of missing structural parameter training, add hyperparameter training for classical parameters in order to find best candidate on cluster
</commit_message>
<xml_diff>
--- a/doc/HyperParameters.xlsx
+++ b/doc/HyperParameters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\papyrus\uni\papyrus_master\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF5703F6-C8EB-41CA-85DF-7EDCDB8724E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{863EFC91-642C-4612-8082-6CD9419AE27F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2F31703B-80AB-4B33-A473-064842AE7FDA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2F31703B-80AB-4B33-A473-064842AE7FDA}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>

</xml_diff>